<commit_message>
Update Project 1 monthly outputs
</commit_message>
<xml_diff>
--- a/Project_1_May2026_Update.xlsx
+++ b/Project_1_May2026_Update.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LSQ_Returns" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SP500TR_Returns" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NVIDIA_Returns" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Updated_Table_2" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Updated_Table_4" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regression" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Serial_Correlation" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Newey_West" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="LSQ_Returns" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="SP500TR_Returns" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="NVIDIA_Returns" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Verification" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Updated_Table_2" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Updated_Table_4" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Regression" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Serial_Correlation" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Newey_West" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -426,7 +426,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="59" customWidth="1" min="2" max="2"/>
+    <col width="53" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -473,7 +473,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>project1_may2026_deliverables\data\LSQ_latest_spartan.pdf</t>
+          <t>data/LSQ_latest_spartan.pdf</t>
         </is>
       </c>
     </row>
@@ -485,7 +485,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-06-12T02:01:28</t>
+          <t>2026-06-12T16:40:04</t>
         </is>
       </c>
     </row>
@@ -4131,7 +4131,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.02285956720180793</v>
+        <v>0.02285929685021193</v>
       </c>
     </row>
     <row r="3">
@@ -4146,7 +4146,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>-0.07052604356294512</v>
+        <v>-0.07052562470952384</v>
       </c>
     </row>
     <row r="4">
@@ -4161,7 +4161,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.07476805121952501</v>
+        <v>0.07476813959401474</v>
       </c>
     </row>
     <row r="5">
@@ -4176,7 +4176,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>-0.04250421583286856</v>
+        <v>-0.04250447489194809</v>
       </c>
     </row>
     <row r="6">
@@ -4191,7 +4191,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.3839884098304449</v>
+        <v>0.3839885382872792</v>
       </c>
     </row>
     <row r="7">
@@ -4206,7 +4206,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.002509417020269522</v>
+        <v>0.002509685278008655</v>
       </c>
     </row>
     <row r="8">
@@ -4221,7 +4221,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.1241703906311096</v>
+        <v>0.1241695546462829</v>
       </c>
     </row>
     <row r="9">
@@ -4236,7 +4236,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.042642832566262</v>
+        <v>0.04264380498718268</v>
       </c>
     </row>
     <row r="10">
@@ -4251,7 +4251,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.05599341871636443</v>
+        <v>0.05599305070825578</v>
       </c>
     </row>
     <row r="11">
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.15684926079897</v>
+        <v>0.1568492438443789</v>
       </c>
     </row>
     <row r="12">
@@ -4281,7 +4281,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>-0.02949579108762135</v>
+        <v>-0.02949597520951819</v>
       </c>
     </row>
     <row r="13">
@@ -4296,7 +4296,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>-0.03525258070522685</v>
+        <v>-0.03525248782048929</v>
       </c>
     </row>
     <row r="14">
@@ -4311,7 +4311,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.2702840449401422</v>
+        <v>0.2702843443308522</v>
       </c>
     </row>
     <row r="15">
@@ -4326,7 +4326,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>-0.01545940462696405</v>
+        <v>-0.01545979379661466</v>
       </c>
     </row>
     <row r="16">
@@ -4341,7 +4341,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>-0.042422091310234</v>
+        <v>-0.04242177889535137</v>
       </c>
     </row>
     <row r="17">
@@ -4356,7 +4356,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>-0.02888714967079109</v>
+        <v>-0.02888722818772815</v>
       </c>
     </row>
     <row r="18">
@@ -4371,7 +4371,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.1213427060924364</v>
+        <v>0.1213426956799988</v>
       </c>
     </row>
     <row r="19">
@@ -4386,7 +4386,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>-0.06004776811367074</v>
+        <v>-0.06004776351854657</v>
       </c>
     </row>
     <row r="20">
@@ -4401,7 +4401,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.0336005150522356</v>
+        <v>0.03360075655618111</v>
       </c>
     </row>
     <row r="21">
@@ -4416,7 +4416,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.1462879444147493</v>
+        <v>0.1462871894254973</v>
       </c>
     </row>
     <row r="22">
@@ -4431,7 +4431,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.001758746802028588</v>
+        <v>0.001759297122216452</v>
       </c>
     </row>
     <row r="23">
@@ -4446,7 +4446,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>-0.2497686501646835</v>
+        <v>-0.2497686673607447</v>
       </c>
     </row>
     <row r="24">
@@ -4461,7 +4461,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>-0.2248255762550559</v>
+        <v>-0.2248259008642258</v>
       </c>
     </row>
     <row r="25">
@@ -4476,7 +4476,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>-0.182319165739989</v>
+        <v>-0.1823190318263749</v>
       </c>
     </row>
     <row r="26">
@@ -4491,7 +4491,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>0.07677896314296184</v>
+        <v>0.07677889655705639</v>
       </c>
     </row>
     <row r="27">
@@ -4506,7 +4506,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0.07311310865577525</v>
+        <v>0.07311291750783333</v>
       </c>
     </row>
     <row r="28">
@@ -4521,7 +4521,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>0.1652080591136154</v>
+        <v>0.1652085475935621</v>
       </c>
     </row>
     <row r="29">
@@ -4536,7 +4536,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>0.008019905667705052</v>
+        <v>0.008020011943399297</v>
       </c>
     </row>
     <row r="30">
@@ -4551,7 +4551,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>-0.2516023421696284</v>
+        <v>-0.2516024481115456</v>
       </c>
     </row>
     <row r="31">
@@ -4566,7 +4566,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>0.2137715849809971</v>
+        <v>0.2137713567816002</v>
       </c>
     </row>
     <row r="32">
@@ -4581,7 +4581,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>0.02733957678342636</v>
+        <v>0.02733934597857735</v>
       </c>
     </row>
     <row r="33">
@@ -4596,7 +4596,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>-0.007171650506887617</v>
+        <v>-0.00717119740444272</v>
       </c>
     </row>
     <row r="34">
@@ -4611,7 +4611,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>0.04019053924864879</v>
+        <v>0.04019030521676048</v>
       </c>
     </row>
     <row r="35">
@@ -4626,7 +4626,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>0.1548228494725041</v>
+        <v>0.1548226459888284</v>
       </c>
     </row>
     <row r="36">
@@ -4641,7 +4641,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>0.07820089684145959</v>
+        <v>0.07820120572670053</v>
       </c>
     </row>
     <row r="37">
@@ -4656,7 +4656,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>0.08643395566166379</v>
+        <v>0.086433778525842</v>
       </c>
     </row>
     <row r="38">
@@ -4671,7 +4671,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>0.004802033998286603</v>
+        <v>0.00480219782459379</v>
       </c>
     </row>
     <row r="39">
@@ -4686,7 +4686,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>0.1422831798125233</v>
+        <v>0.1422832609445948</v>
       </c>
     </row>
     <row r="40">
@@ -4701,7 +4701,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>-0.02337295768505621</v>
+        <v>-0.02337295602496314</v>
       </c>
     </row>
     <row r="41">
@@ -4716,7 +4716,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>0.1088013073235865</v>
+        <v>0.1088010812327445</v>
       </c>
     </row>
     <row r="42">
@@ -4731,7 +4731,7 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>0.2146567229905958</v>
+        <v>0.2146575382268885</v>
       </c>
     </row>
     <row r="43">
@@ -4746,7 +4746,7 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>0.07010912259352398</v>
+        <v>0.07010843675235567</v>
       </c>
     </row>
     <row r="44">
@@ -4761,7 +4761,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>0.1181168732147577</v>
+        <v>0.1181168851353178</v>
       </c>
     </row>
     <row r="45">
@@ -4776,7 +4776,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>0.2599918765598133</v>
+        <v>0.2599920805477076</v>
       </c>
     </row>
     <row r="46">
@@ -4791,7 +4791,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>0.01166416049041263</v>
+        <v>0.01166394474764676</v>
       </c>
     </row>
     <row r="47">
@@ -4806,7 +4806,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>-0.07337155693543396</v>
+        <v>-0.07337114246742593</v>
       </c>
     </row>
     <row r="48">
@@ -4821,7 +4821,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>0.06921181850047553</v>
+        <v>0.06921179734475302</v>
       </c>
     </row>
     <row r="49">
@@ -4836,7 +4836,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>-0.02585514253340404</v>
+        <v>-0.02585556396201738</v>
       </c>
     </row>
     <row r="50">
@@ -4851,7 +4851,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>-0.004704362017168506</v>
+        <v>-0.004704069239626296</v>
       </c>
     </row>
     <row r="51">
@@ -4866,7 +4866,7 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>0.05579406449729629</v>
+        <v>0.05579405627172118</v>
       </c>
     </row>
     <row r="52">
@@ -4881,7 +4881,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>-0.02670521194141107</v>
+        <v>-0.02670541766719159</v>
       </c>
     </row>
     <row r="53">
@@ -4896,7 +4896,7 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>0.1248425350174647</v>
+        <v>0.1248426157068663</v>
       </c>
     </row>
     <row r="54">
@@ -4911,7 +4911,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>0.08228136449543633</v>
+        <v>0.08228110940569455</v>
       </c>
     </row>
     <row r="55">
@@ -4926,7 +4926,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>0.2313400691415173</v>
+        <v>0.2313404772121077</v>
       </c>
     </row>
     <row r="56">
@@ -4941,7 +4941,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>-0.02494877269816898</v>
+        <v>-0.02494867460315708</v>
       </c>
     </row>
     <row r="57">
@@ -4956,7 +4956,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>0.1480076467541931</v>
+        <v>0.1480073232301915</v>
       </c>
     </row>
     <row r="58">
@@ -4971,7 +4971,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>-0.07439577103852923</v>
+        <v>-0.07439560639689813</v>
       </c>
     </row>
     <row r="59">
@@ -4986,7 +4986,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>0.2341670254606225</v>
+        <v>0.2341669114563416</v>
       </c>
     </row>
     <row r="60">
@@ -5001,7 +5001,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>0.2780538211469497</v>
+        <v>0.278053372066061</v>
       </c>
     </row>
     <row r="61">
@@ -5016,7 +5016,7 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>-0.09992038929948788</v>
+        <v>-0.0999201901568485</v>
       </c>
     </row>
     <row r="62">
@@ -5031,7 +5031,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>-0.1673525319215579</v>
+        <v>-0.1673522934414061</v>
       </c>
     </row>
     <row r="63">
@@ -5046,7 +5046,7 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>-0.004124780510119108</v>
+        <v>-0.004125014290136009</v>
       </c>
     </row>
     <row r="64">
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>0.1189665252488112</v>
+        <v>0.1189666130487661</v>
       </c>
     </row>
     <row r="65">
@@ -5076,7 +5076,7 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>-0.3201581692865763</v>
+        <v>-0.3201583796553739</v>
       </c>
     </row>
     <row r="66">
@@ -5091,7 +5091,7 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>0.006739453326456868</v>
+        <v>0.006739971141816792</v>
       </c>
     </row>
     <row r="67">
@@ -5106,7 +5106,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>-0.188142645455245</v>
+        <v>-0.1881427605859263</v>
       </c>
     </row>
     <row r="68">
@@ -5121,7 +5121,7 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>0.1984195361864451</v>
+        <v>0.1984193343680376</v>
       </c>
     </row>
     <row r="69">
@@ -5136,7 +5136,7 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>-0.168969954550624</v>
+        <v>-0.1689698670395005</v>
       </c>
     </row>
     <row r="70">
@@ -5151,7 +5151,7 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>-0.1957732395604797</v>
+        <v>-0.1957731128449735</v>
       </c>
     </row>
     <row r="71">
@@ -5166,7 +5166,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>0.1122013345021275</v>
+        <v>0.1122011592615861</v>
       </c>
     </row>
     <row r="72">
@@ -5181,7 +5181,7 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>0.2538340326238617</v>
+        <v>0.2538341742905792</v>
       </c>
     </row>
     <row r="73">
@@ -5196,7 +5196,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>-0.136220466658155</v>
+        <v>-0.1362205642538448</v>
       </c>
     </row>
     <row r="74">
@@ -5211,7 +5211,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>0.3368686043227049</v>
+        <v>0.3368688659330197</v>
       </c>
     </row>
     <row r="75">
@@ -5226,7 +5226,7 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>0.1883094486906212</v>
+        <v>0.1883092161517261</v>
       </c>
     </row>
     <row r="76">
@@ -5256,7 +5256,7 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>-0.0008382849217655197</v>
+        <v>-0.0008381472836533899</v>
       </c>
     </row>
     <row r="78">
@@ -5271,7 +5271,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>0.363436671024731</v>
+        <v>0.3634366209600322</v>
       </c>
     </row>
     <row r="79">
@@ -5286,7 +5286,7 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>0.1180947111783819</v>
+        <v>0.1180945982127071</v>
       </c>
     </row>
     <row r="80">
@@ -5316,7 +5316,7 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>0.05619639406771304</v>
+        <v>0.05619647586122234</v>
       </c>
     </row>
     <row r="82">
@@ -5331,7 +5331,7 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>-0.1186506332668394</v>
+        <v>-0.1186507015199146</v>
       </c>
     </row>
     <row r="83">
@@ -5346,7 +5346,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>-0.0624297173404752</v>
+        <v>-0.0624299809416361</v>
       </c>
     </row>
     <row r="84">
@@ -5361,7 +5361,7 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>0.146885644002696</v>
+        <v>0.1468857790179774</v>
       </c>
     </row>
     <row r="85">
@@ -5376,7 +5376,7 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>0.05884105488915115</v>
+        <v>0.05884106450555349</v>
       </c>
     </row>
     <row r="86">
@@ -5391,7 +5391,7 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>0.2425268114256502</v>
+        <v>0.2425270032073543</v>
       </c>
     </row>
     <row r="87">
@@ -5406,7 +5406,7 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>0.2858093415179341</v>
+        <v>0.2858092172967774</v>
       </c>
     </row>
     <row r="88">
@@ -5421,7 +5421,7 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>0.1421276597389094</v>
+        <v>0.1421278666884103</v>
       </c>
     </row>
     <row r="89">
@@ -5436,7 +5436,7 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>-0.04371539540089564</v>
+        <v>-0.04371539170313565</v>
       </c>
     </row>
     <row r="90">
@@ -5451,7 +5451,7 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>0.2688711393283107</v>
+        <v>0.2688710270916701</v>
       </c>
     </row>
     <row r="91">
@@ -5481,7 +5481,7 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>-0.05269877881153473</v>
+        <v>-0.05269871694819739</v>
       </c>
     </row>
     <row r="93">
@@ -5496,7 +5496,7 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>0.02008221224001749</v>
+        <v>0.02008208031891745</v>
       </c>
     </row>
     <row r="94">
@@ -5511,7 +5511,7 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>0.01734106599608709</v>
+        <v>0.01734106710624794</v>
       </c>
     </row>
     <row r="95">
@@ -5526,7 +5526,7 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>0.09330822424722918</v>
+        <v>0.09330816719098234</v>
       </c>
     </row>
     <row r="96">
@@ -5541,7 +5541,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>0.04135289270640019</v>
+        <v>0.04135312769620292</v>
       </c>
     </row>
     <row r="97">
@@ -5556,7 +5556,7 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>-0.02864379346153278</v>
+        <v>-0.02864401138199291</v>
       </c>
     </row>
     <row r="98">
@@ -5571,7 +5571,7 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>-0.1058287148205893</v>
+        <v>-0.1058285561594333</v>
       </c>
     </row>
     <row r="99">
@@ -5586,7 +5586,7 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>0.04039309306242167</v>
+        <v>0.04039296321972285</v>
       </c>
     </row>
     <row r="100">
@@ -5601,7 +5601,7 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>-0.1324047519202285</v>
+        <v>-0.1324046988533616</v>
       </c>
     </row>
     <row r="101">
@@ -5646,7 +5646,7 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>0.16917037363203</v>
+        <v>0.1691704867095978</v>
       </c>
     </row>
     <row r="104">
@@ -5661,7 +5661,7 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>0.1259088530315122</v>
+        <v>0.1259087441380393</v>
       </c>
     </row>
     <row r="105">
@@ -5676,7 +5676,7 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>-0.02074555918313137</v>
+        <v>-0.02074547328268472</v>
       </c>
     </row>
     <row r="106">
@@ -5691,7 +5691,7 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>0.07119086207604353</v>
+        <v>0.07119068039067433</v>
       </c>
     </row>
     <row r="107">
@@ -5706,7 +5706,7 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>0.08533291274421861</v>
+        <v>0.08533300162257662</v>
       </c>
     </row>
     <row r="108">
@@ -6273,7 +6273,7 @@
         <v>3.495221238938055</v>
       </c>
       <c r="C2" t="n">
-        <v>4.847036963910896</v>
+        <v>4.847037080431163</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -6291,7 +6291,7 @@
         <v>3.422856966733567</v>
       </c>
       <c r="C3" t="n">
-        <v>3.957808638228077</v>
+        <v>3.957808721770739</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -6345,7 +6345,7 @@
         <v>3.697222222222224</v>
       </c>
       <c r="C6" t="n">
-        <v>12.37256045848575</v>
+        <v>12.37256016259983</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -6363,7 +6363,7 @@
         <v>-0.8680000000000002</v>
       </c>
       <c r="C7" t="n">
-        <v>-8.887043413688216</v>
+        <v>-8.887042544526659</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -6381,7 +6381,7 @@
         <v>21.97</v>
       </c>
       <c r="C8" t="n">
-        <v>38.39884098304449</v>
+        <v>38.39885382872792</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -6399,7 +6399,7 @@
         <v>-2.2</v>
       </c>
       <c r="C9" t="n">
-        <v>-32.01581692865763</v>
+        <v>-32.01583796553739</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -6417,7 +6417,7 @@
         <v>3.495221238938055</v>
       </c>
       <c r="C10" t="n">
-        <v>4.847036963910896</v>
+        <v>4.847037080431163</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -6435,7 +6435,7 @@
         <v>3.992318974200495</v>
       </c>
       <c r="C11" t="n">
-        <v>13.47440125568114</v>
+        <v>13.47440142378295</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -6453,7 +6453,7 @@
         <v>2.614250975720806</v>
       </c>
       <c r="C12" t="n">
-        <v>-0.04823758466202541</v>
+        <v>-0.0482374382237372</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -6471,7 +6471,7 @@
         <v>8.093367320642244</v>
       </c>
       <c r="C13" t="n">
-        <v>0.06682697879962607</v>
+        <v>0.06682952564226774</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -6489,7 +6489,7 @@
         <v>0.8754864682719924</v>
       </c>
       <c r="C14" t="n">
-        <v>0.359721880916027</v>
+        <v>0.3597218850757939</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -6507,7 +6507,7 @@
         <v>14.35776078315886</v>
       </c>
       <c r="C15" t="n">
-        <v>0.6802039332048143</v>
+        <v>0.6802039139380652</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -6525,7 +6525,7 @@
         <v>92.0046082949309</v>
       </c>
       <c r="C16" t="n">
-        <v>2.540768823291434</v>
+        <v>2.540769011019441</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Remove zip artifacts from monthly workspace
</commit_message>
<xml_diff>
--- a/Project_1_May2026_Update.xlsx
+++ b/Project_1_May2026_Update.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="LSQ_Returns" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="SP500TR_Returns" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="NVIDIA_Returns" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Verification" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Updated_Table_2" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Updated_Table_4" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Regression" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Serial_Correlation" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Newey_West" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LSQ_Returns" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SP500TR_Returns" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NVIDIA_Returns" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Updated_Table_2" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Updated_Table_4" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regression" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Serial_Correlation" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Newey_West" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -473,7 +473,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>data/LSQ_latest_spartan.pdf</t>
+          <t>data\LSQ_latest_spartan.pdf</t>
         </is>
       </c>
     </row>
@@ -485,7 +485,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-06-12T19:20:04</t>
+          <t>2026-06-12T15:23:43</t>
         </is>
       </c>
     </row>
@@ -4131,7 +4131,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.02285947846851455</v>
+        <v>0.02285966216268376</v>
       </c>
     </row>
     <row r="3">
@@ -4146,7 +4146,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>-0.07052561218703712</v>
+        <v>-0.0705258722648533</v>
       </c>
     </row>
     <row r="4">
@@ -4161,7 +4161,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.07476793427886541</v>
+        <v>0.07476823511005271</v>
       </c>
     </row>
     <row r="5">
@@ -4176,7 +4176,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>-0.0425041194067628</v>
+        <v>-0.04250438224323216</v>
       </c>
     </row>
     <row r="6">
@@ -4191,7 +4191,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.3839884885419578</v>
+        <v>0.3839886526392016</v>
       </c>
     </row>
     <row r="7">
@@ -4206,7 +4206,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.002509416178806623</v>
+        <v>0.002509148089431923</v>
       </c>
     </row>
     <row r="8">
@@ -4221,7 +4221,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.1241696132363102</v>
+        <v>0.1241705244242364</v>
       </c>
     </row>
     <row r="9">
@@ -4236,7 +4236,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.04264391892696051</v>
+        <v>0.04264294650610112</v>
       </c>
     </row>
     <row r="10">
@@ -4251,7 +4251,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.0559926954833152</v>
+        <v>0.05599317763857115</v>
       </c>
     </row>
     <row r="11">
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.15684926079897</v>
+        <v>0.1568494769886124</v>
       </c>
     </row>
     <row r="12">
@@ -4281,7 +4281,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>-0.02949588452660679</v>
+        <v>-0.02949597245344471</v>
       </c>
     </row>
     <row r="13">
@@ -4296,7 +4296,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>-0.03525219898404675</v>
+        <v>-0.03525258070522685</v>
       </c>
     </row>
     <row r="14">
@@ -4311,7 +4311,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.2702839640196344</v>
+        <v>0.2702840449401422</v>
       </c>
     </row>
     <row r="15">
@@ -4326,7 +4326,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>-0.01545955810866706</v>
+        <v>-0.01545971887763486</v>
       </c>
     </row>
     <row r="16">
@@ -4341,7 +4341,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>-0.04242192833258129</v>
+        <v>-0.04242178566555299</v>
       </c>
     </row>
     <row r="17">
@@ -4356,7 +4356,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>-0.02888722578051672</v>
+        <v>-0.0288869830080688</v>
       </c>
     </row>
     <row r="18">
@@ -4371,7 +4371,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.1213427710777206</v>
+        <v>0.121342685267563</v>
       </c>
     </row>
     <row r="19">
@@ -4386,7 +4386,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>-0.06004806042616784</v>
+        <v>-0.06004814154578675</v>
       </c>
     </row>
     <row r="20">
@@ -4401,7 +4401,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.03360059920092984</v>
+        <v>0.03360093032472533</v>
       </c>
     </row>
     <row r="21">
@@ -4416,7 +4416,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.1462877868816175</v>
+        <v>0.14628737000368</v>
       </c>
     </row>
     <row r="22">
@@ -4431,7 +4431,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.001759021901640123</v>
+        <v>0.001759159693233814</v>
       </c>
     </row>
     <row r="23">
@@ -4446,7 +4446,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>-0.2497688216809697</v>
+        <v>-0.2497685644382728</v>
       </c>
     </row>
     <row r="24">
@@ -4461,7 +4461,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>-0.2248255968109131</v>
+        <v>-0.2248259008642258</v>
       </c>
     </row>
     <row r="25">
@@ -4476,7 +4476,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>-0.182319128270181</v>
+        <v>-0.1823190908003643</v>
       </c>
     </row>
     <row r="26">
@@ -4491,7 +4491,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>0.07677882443358564</v>
+        <v>0.07677890209461724</v>
       </c>
     </row>
     <row r="27">
@@ -4506,7 +4506,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0.07311319032805774</v>
+        <v>0.07311298938575894</v>
       </c>
     </row>
     <row r="28">
@@ -4521,7 +4521,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>0.1652083294062485</v>
+        <v>0.1652084227590536</v>
       </c>
     </row>
     <row r="29">
@@ -4536,7 +4536,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>0.008019904808493239</v>
+        <v>0.008019691397869622</v>
       </c>
     </row>
     <row r="30">
@@ -4551,7 +4551,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>-0.2516023685699601</v>
+        <v>-0.2516020768038197</v>
       </c>
     </row>
     <row r="31">
@@ -4566,7 +4566,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>0.2137713567816002</v>
+        <v>0.2137712705956767</v>
       </c>
     </row>
     <row r="32">
@@ -4581,7 +4581,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>0.0273394629803918</v>
+        <v>0.02733969698402072</v>
       </c>
     </row>
     <row r="33">
@@ -4596,7 +4596,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>-0.007171538252247034</v>
+        <v>-0.0071719921713288</v>
       </c>
     </row>
     <row r="34">
@@ -4611,7 +4611,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>0.04019042914811277</v>
+        <v>0.04019055307952191</v>
       </c>
     </row>
     <row r="35">
@@ -4626,7 +4626,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>0.1548228836198227</v>
+        <v>0.1548226801361059</v>
       </c>
     </row>
     <row r="36">
@@ -4641,7 +4641,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>0.07820129375297236</v>
+        <v>0.07820150714433938</v>
       </c>
     </row>
     <row r="37">
@@ -4656,7 +4656,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>0.08643349751164076</v>
+        <v>0.08643350516687431</v>
       </c>
     </row>
     <row r="38">
@@ -4671,7 +4671,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>0.004802361259457877</v>
+        <v>0.00480244317265166</v>
       </c>
     </row>
     <row r="39">
@@ -4686,7 +4686,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>0.1422834116649898</v>
+        <v>0.1422832494008599</v>
       </c>
     </row>
     <row r="40">
@@ -4701,7 +4701,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>-0.02337309309711155</v>
+        <v>-0.02337281231242416</v>
       </c>
     </row>
     <row r="41">
@@ -4716,7 +4716,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>0.1088012187721632</v>
+        <v>0.1088009847686955</v>
       </c>
     </row>
     <row r="42">
@@ -4731,7 +4731,7 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>0.2146569056806928</v>
+        <v>0.2146569853497966</v>
       </c>
     </row>
     <row r="43">
@@ -4746,7 +4746,7 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>0.07010878345862448</v>
+        <v>0.07010899945310189</v>
       </c>
     </row>
     <row r="44">
@@ -4761,7 +4761,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>0.1181167842135795</v>
+        <v>0.1181163566856096</v>
       </c>
     </row>
     <row r="45">
@@ -4776,7 +4776,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>0.2599922845356388</v>
+        <v>0.2599924217301743</v>
       </c>
     </row>
     <row r="46">
@@ -4791,7 +4791,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>0.01166380064063821</v>
+        <v>0.01166423129057348</v>
       </c>
     </row>
     <row r="47">
@@ -4806,7 +4806,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>-0.07337114766282293</v>
+        <v>-0.07337161735437492</v>
       </c>
     </row>
     <row r="48">
@@ -4821,7 +4821,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>0.06921134413415575</v>
+        <v>0.06921196604474256</v>
       </c>
     </row>
     <row r="49">
@@ -4836,7 +4836,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>-0.02585514807700895</v>
+        <v>-0.02585527992983927</v>
       </c>
     </row>
     <row r="50">
@@ -4851,7 +4851,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>-0.004703922850822995</v>
+        <v>-0.004704361672023816</v>
       </c>
     </row>
     <row r="51">
@@ -4866,7 +4866,7 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>0.0557940521589344</v>
+        <v>0.0557940603845084</v>
       </c>
     </row>
     <row r="52">
@@ -4881,7 +4881,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>-0.02670520634787643</v>
+        <v>-0.02670534971344485</v>
       </c>
     </row>
     <row r="53">
@@ -4896,7 +4896,7 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>0.1248423646832617</v>
+        <v>0.1248426157068663</v>
       </c>
     </row>
     <row r="54">
@@ -4911,7 +4911,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>0.08228142302058505</v>
+        <v>0.08228098186082344</v>
       </c>
     </row>
     <row r="55">
@@ -4926,7 +4926,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>0.2313394526377714</v>
+        <v>0.2313400330823481</v>
       </c>
     </row>
     <row r="56">
@@ -4941,7 +4941,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>-0.02494820800560771</v>
+        <v>-0.02494830371288737</v>
       </c>
     </row>
     <row r="57">
@@ -4956,7 +4956,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>0.1480076176984868</v>
+        <v>0.1480076322263386</v>
       </c>
     </row>
     <row r="58">
@@ -4971,7 +4971,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>-0.07439584381792541</v>
+        <v>-0.07439567917632861</v>
       </c>
     </row>
     <row r="59">
@@ -4986,7 +4986,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>0.2341670038298038</v>
+        <v>0.2341667974520816</v>
       </c>
     </row>
     <row r="60">
@@ -5001,7 +5001,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>0.2780534261014624</v>
+        <v>0.2780539708405791</v>
       </c>
     </row>
     <row r="61">
@@ -5016,7 +5016,7 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>-0.09992041270609098</v>
+        <v>-0.09992061184862888</v>
       </c>
     </row>
     <row r="62">
@@ -5031,7 +5031,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>-0.1673522501543653</v>
+        <v>-0.1673523585057887</v>
       </c>
     </row>
     <row r="63">
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>0.1189665252488112</v>
+        <v>0.1189666821792394</v>
       </c>
     </row>
     <row r="65">
@@ -5076,7 +5076,7 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>-0.3201582394095088</v>
+        <v>-0.3201581243857232</v>
       </c>
     </row>
     <row r="66">
@@ -5091,7 +5091,7 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>0.006739557167566579</v>
+        <v>0.00673914249837182</v>
       </c>
     </row>
     <row r="67">
@@ -5106,7 +5106,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>-0.1881425429997872</v>
+        <v>-0.1881426135037536</v>
       </c>
     </row>
     <row r="68">
@@ -5121,7 +5121,7 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>0.1984192587484812</v>
+        <v>0.1984196118060286</v>
       </c>
     </row>
     <row r="69">
@@ -5136,7 +5136,7 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>-0.1689699723439044</v>
+        <v>-0.1689700072028205</v>
       </c>
     </row>
     <row r="70">
@@ -5151,7 +5151,7 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>-0.1957730742947046</v>
+        <v>-0.1957731252487188</v>
       </c>
     </row>
     <row r="71">
@@ -5166,7 +5166,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>0.1122011681009001</v>
+        <v>0.1122010893199503</v>
       </c>
     </row>
     <row r="72">
@@ -5181,7 +5181,7 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>0.2538345464373262</v>
+        <v>0.2538342102504385</v>
       </c>
     </row>
     <row r="73">
@@ -5196,7 +5196,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>-0.1362208159385478</v>
+        <v>-0.136220466658155</v>
       </c>
     </row>
     <row r="74">
@@ -5211,7 +5211,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>0.3368690841728628</v>
+        <v>0.3368687351278623</v>
       </c>
     </row>
     <row r="75">
@@ -5226,7 +5226,7 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>0.1883090998823127</v>
+        <v>0.1883092345767339</v>
       </c>
     </row>
     <row r="76">
@@ -5241,7 +5241,7 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>0.1964592501287579</v>
+        <v>0.1964593486442521</v>
       </c>
     </row>
     <row r="77">
@@ -5271,7 +5271,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>0.3634363955175532</v>
+        <v>0.363436671024731</v>
       </c>
     </row>
     <row r="79">
@@ -5286,7 +5286,7 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>0.1180949371097999</v>
+        <v>0.1180945091101937</v>
       </c>
     </row>
     <row r="80">
@@ -5301,7 +5301,7 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>0.1047664624860469</v>
+        <v>0.1047668428710162</v>
       </c>
     </row>
     <row r="81">
@@ -5316,7 +5316,7 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>0.05619648045772951</v>
+        <v>0.05619630767771078</v>
       </c>
     </row>
     <row r="82">
@@ -5331,7 +5331,7 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>-0.1186505558252673</v>
+        <v>-0.1186507107084115</v>
       </c>
     </row>
     <row r="83">
@@ -5346,7 +5346,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>-0.06243006332314394</v>
+        <v>-0.06242972282599102</v>
       </c>
     </row>
     <row r="84">
@@ -5361,7 +5361,7 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>0.1468858727358351</v>
+        <v>0.1468857514863415</v>
       </c>
     </row>
     <row r="85">
@@ -5376,7 +5376,7 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>0.05884114141242036</v>
+        <v>0.05884105488915115</v>
       </c>
     </row>
     <row r="86">
@@ -5391,7 +5391,7 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>0.2425266570775326</v>
+        <v>0.2425267342515915</v>
       </c>
     </row>
     <row r="87">
@@ -5406,7 +5406,7 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>0.2858097496850216</v>
+        <v>0.2858096698226296</v>
       </c>
     </row>
     <row r="88">
@@ -5436,7 +5436,7 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>-0.04371531081375535</v>
+        <v>-0.04371522622661506</v>
       </c>
     </row>
     <row r="90">
@@ -5451,7 +5451,7 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>0.2688710270916701</v>
+        <v>0.2688710033089727</v>
       </c>
     </row>
     <row r="91">
@@ -5466,7 +5466,7 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>0.1268505324471054</v>
+        <v>0.1268503841828028</v>
       </c>
     </row>
     <row r="92">
@@ -5481,7 +5481,7 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>-0.05269871694819739</v>
+        <v>-0.052698658344975</v>
       </c>
     </row>
     <row r="93">
@@ -5496,7 +5496,7 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>0.02008208031891745</v>
+        <v>0.02008214562373478</v>
       </c>
     </row>
     <row r="94">
@@ -5511,7 +5511,7 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>0.01734113112542701</v>
+        <v>0.01734106599608709</v>
       </c>
     </row>
     <row r="95">
@@ -5526,7 +5526,7 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>0.09330797253547929</v>
+        <v>0.09330822424722918</v>
       </c>
     </row>
     <row r="96">
@@ -5541,7 +5541,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>0.04135301734180707</v>
+        <v>0.04135289270640019</v>
       </c>
     </row>
     <row r="97">
@@ -5556,7 +5556,7 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>-0.02864379662791638</v>
+        <v>-0.02864379346153278</v>
       </c>
     </row>
     <row r="98">
@@ -5571,7 +5571,7 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>-0.1058286130610341</v>
+        <v>-0.1058287148205893</v>
       </c>
     </row>
     <row r="99">
@@ -5736,7 +5736,7 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>0.05367232174856373</v>
+        <v>0.05367240806636397</v>
       </c>
     </row>
     <row r="110">
@@ -5751,7 +5751,7 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>0.02488282237211026</v>
+        <v>0.02488273841277922</v>
       </c>
     </row>
     <row r="111">
@@ -6237,7 +6237,7 @@
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -6273,7 +6273,7 @@
         <v>3.495221238938055</v>
       </c>
       <c r="C2" t="n">
-        <v>4.847036853460228</v>
+        <v>4.847037161994041</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -6291,7 +6291,7 @@
         <v>3.422856966733567</v>
       </c>
       <c r="C3" t="n">
-        <v>3.957808721770739</v>
+        <v>3.957808805313401</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -6345,7 +6345,7 @@
         <v>3.697222222222224</v>
       </c>
       <c r="C6" t="n">
-        <v>12.37255821599764</v>
+        <v>12.37256091799214</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -6363,7 +6363,7 @@
         <v>-0.8680000000000002</v>
       </c>
       <c r="C7" t="n">
-        <v>-8.887039633170533</v>
+        <v>-8.887043692702484</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -6381,7 +6381,7 @@
         <v>21.97</v>
       </c>
       <c r="C8" t="n">
-        <v>38.39884885419578</v>
+        <v>38.39886526392016</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -6399,7 +6399,7 @@
         <v>-2.2</v>
       </c>
       <c r="C9" t="n">
-        <v>-32.01582394095088</v>
+        <v>-32.01581243857233</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -6417,7 +6417,7 @@
         <v>3.495221238938055</v>
       </c>
       <c r="C10" t="n">
-        <v>4.847036853460228</v>
+        <v>4.847037161994041</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -6435,7 +6435,7 @@
         <v>3.992318974200495</v>
       </c>
       <c r="C11" t="n">
-        <v>13.47439979390154</v>
+        <v>13.4744020813298</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -6453,7 +6453,7 @@
         <v>2.614250975720806</v>
       </c>
       <c r="C12" t="n">
-        <v>-0.048237383625256</v>
+        <v>-0.04823653960140341</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -6471,7 +6471,7 @@
         <v>8.093367320642244</v>
       </c>
       <c r="C13" t="n">
-        <v>0.06682923659618512</v>
+        <v>0.06682762078836069</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -6489,7 +6489,7 @@
         <v>0.8754864682719924</v>
       </c>
       <c r="C14" t="n">
-        <v>0.3597219117436294</v>
+        <v>0.3597218735746442</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -6507,7 +6507,7 @@
         <v>14.35776078315886</v>
       </c>
       <c r="C15" t="n">
-        <v>0.6802039762800973</v>
+        <v>0.6802040455549085</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -6525,7 +6525,7 @@
         <v>92.0046082949309</v>
       </c>
       <c r="C16" t="n">
-        <v>2.540769443619561</v>
+        <v>2.540768837884408</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>

</xml_diff>